<commit_message>
commit Aloïs 16h09 19/06
</commit_message>
<xml_diff>
--- a/data/output/Garches_Equipe_1_feuille.xlsx
+++ b/data/output/Garches_Equipe_1_feuille.xlsx
@@ -498,7 +498,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
@@ -528,7 +528,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
@@ -558,7 +558,7 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>

</xml_diff>

<commit_message>
Main fonctionnel avec generation de l'excell des P M 14h52 22/06/2026 Rayane et Thibaut
</commit_message>
<xml_diff>
--- a/data/output/Garches_Equipe_1_feuille.xlsx
+++ b/data/output/Garches_Equipe_1_feuille.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,12 +469,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>48.838467608,2.171797485</t>
+          <t>48.842130147,2.187364881</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Allée  de  la  Marc he  /  Boulevard  Raymond  Poincaré  D907</t>
+          <t>Avenue  de  Lorraine  /  Avenue  d'Alsace</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -494,12 +494,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>48.838467608,2.171797485</t>
+          <t>48.842130147,2.187364881</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Allée  de  la  Marc he  /  Boulevard  Raymond  Poincaré  D907</t>
+          <t>Avenue  de  Lorraine  /  Avenue  d'Alsace</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -519,19 +519,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>48.838467608,2.171797485</t>
+          <t>48.842677932,2.186438811</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Allée  de  la  Marc he  /  Boulevard  Raymond  Poincaré  D907</t>
+          <t>Avenue  d'Alsace  /  Avenue  Foch / Avenue  d'Alsace  /  Jardin  de  la  Mairie / Avenue  d'Alsace  /  Rue  Georges  Clemenceau / Avenue  Foch  /  Avenue   du  Maréchal  Leclerc / Avenue  Foch  /  Jardin  de  la  Mairie / Avenue  Foch  /  Rue  de  l'Abreuvoir / Jardin  de  la  Mairie  /  Avenue  Foch / Rue  Georges  Clemenceau  /  Avenue  Foch</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
@@ -544,19 +544,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>48.838467608,2.171797485</t>
+          <t>48.842677932,2.186438811</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Allée  de  la  Marc he  /  Boulevard  Raymond  Poincaré  D907</t>
+          <t>Avenue  d'Alsace  /  Avenue  Foch / Avenue  d'Alsace  /  Jardin  de  la  Mairie / Avenue  d'Alsace  /  Rue  Georges  Clemenceau / Avenue  Foch  /  Avenue   du  Maréchal  Leclerc / Avenue  Foch  /  Jardin  de  la  Mairie / Avenue  Foch  /  Rue  de  l'Abreuvoir / Jardin  de  la  Mairie  /  Avenue  Foch / Rue  Georges  Clemenceau  /  Avenue  Foch</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
@@ -569,19 +569,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>48.839372363,2.171812121</t>
+          <t>48.842677932,2.186438811</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Avenue  de  Brétigny  /  Allée  de  la  Marc he</t>
+          <t>Avenue  d'Alsace  /  Avenue  Foch / Avenue  d'Alsace  /  Jardin  de  la  Mairie / Avenue  d'Alsace  /  Rue  Georges  Clemenceau / Avenue  Foch  /  Avenue   du  Maréchal  Leclerc / Avenue  Foch  /  Jardin  de  la  Mairie / Avenue  Foch  /  Rue  de  l'Abreuvoir / Jardin  de  la  Mairie  /  Avenue  Foch / Rue  Georges  Clemenceau  /  Avenue  Foch</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -594,12 +594,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>48.838040862,2.169032756</t>
+          <t>48.842956926,2.186487926</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Boulevard  Raymond  Poincaré  D907  /  Rue  Yves Cariou  D407</t>
+          <t>Avenue   du  Maréchal  Leclerc  /  Rue  de  l'Abreuvoir / Rue  Claude   Liard  /  Avenue   du  Maréchal  Leclerc</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -619,25 +619,625 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48.837882396,2.168128382</t>
+          <t>48.842956926,2.186487926</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Boulevard  de  la  République  D907  /  Boulevard  Raymond  Poincaré  D907 / Boulevard  Raymond  Poincaré  D907  /  Boulevard  de  la  République  D907</t>
+          <t>Avenue   du  Maréchal  Leclerc  /  Rue  de  l'Abreuvoir / Rue  Claude   Liard  /  Avenue   du  Maréchal  Leclerc</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>48.842956926,2.186487926</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Avenue   du  Maréchal  Leclerc  /  Rue  de  l'Abreuvoir / Rue  Claude   Liard  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>48.842956926,2.186487926</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Avenue   du  Maréchal  Leclerc  /  Rue  de  l'Abreuvoir / Rue  Claude   Liard  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>48.843635567,2.186699047</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Passage  Albert  Lanoe  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>48.843635567,2.186699047</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Passage  Albert  Lanoe  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>48.843635567,2.186699047</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Passage  Albert  Lanoe  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>48.843635567,2.186699047</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Passage  Albert  Lanoe  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>48.844591533,2.186878445</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Avenue   du  Maréchal  Leclerc  /  Grande  Rue  / Grande  Rue   /  Avenue   du  Maréchal  Leclerc / Rue  Athime  Rué  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>48.844591533,2.186878445</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Avenue   du  Maréchal  Leclerc  /  Grande  Rue  / Grande  Rue   /  Avenue   du  Maréchal  Leclerc / Rue  Athime  Rué  /  Avenue   du  Maréchal  Leclerc</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>48.84484698,2.186514003</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Avenue  de  Beauval  /  Place  Charles   Devos</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>48.84484698,2.186514003</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Avenue  de  Beauval  /  Place  Charles   Devos</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>48.845207116,2.184629247</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Avenue  de  Beauval  /  Avenue  des  Coteaux / Avenue  des  Coteaux  /  Avenue  de  Beauval</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>48.845382622,2.183603112</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avenue  de  Beauval  /  Rue  de  L'Ermitage / Avenue  de  Beauval  /  Sente  de  la  Plaine </t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>48.845382622,2.183603112</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avenue  de  Beauval  /  Rue  de  L'Ermitage / Avenue  de  Beauval  /  Sente  de  la  Plaine </t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>48.844292567,2.183697322</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avenue  des  Coteaux  /  Impasse  du  Regard / Avenue  des  Coteaux  /  Sente  de  la  Plaine </t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>9</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>48.843732399,2.183521369</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Rue   du  Regard  /  Avenue  des  Coteaux</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>48.845861542,2.185216473</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Rue  Athime  Rué  /  Avenue  des  Coteaux</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>11</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>48.845861542,2.185216473</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Rue  Athime  Rué  /  Avenue  des  Coteaux</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>11</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>48.845861542,2.185216473</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Rue  Athime  Rué  /  Avenue  des  Coteaux</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>11</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>48.845861542,2.185216473</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rue  Athime  Rué  /  Avenue  des  Coteaux</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>11</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>48.844046988,2.18906415</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avenue  de  Lorraine  /  Grande  Rue </t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>12</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>48.844046988,2.18906415</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Avenue  de  Lorraine  /  Grande  Rue </t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>48.843335056,2.188106937</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Avenue  de  Lorraine  /  Jardin  de  la  Mairie</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>13</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>48.843335056,2.188106937</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Avenue  de  Lorraine  /  Jardin  de  la  Mairie</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>13</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>48.843335056,2.188106937</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Avenue  de  Lorraine  /  Jardin  de  la  Mairie</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>13</v>
+      </c>
+      <c r="E32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>